<commit_message>
docs: sync backlog and external integrations roadmap
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Scrum/13_Release_Plan_CitaJusta.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Scrum/13_Release_Plan_CitaJusta.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="1" r:id="Rb73cf054eb9d48c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen Release" sheetId="2" r:id="R4bcf4cc0b6df49c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="1" r:id="R930de630639949fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen Release" sheetId="2" r:id="Rfb3d5ac6481e4597"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -74,150 +74,78 @@
     <x:t xml:space="preserve">Base documental suficiente para continuar el desarrollo incremental.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">R0.3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sprint 3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Seguridad y usuarios</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Auth, sesiones, JWT, RBAC, contexto institucional y validación</x:t>
+    <x:t xml:space="preserve">R0.4</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sprint 4</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agenda base</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Instituciones, sedes, servicios, profesionales y disponibilidad read-only</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Catálogo institucional, servicios, profesionales y disponibilidad read-only; 69/69 pruebas unitarias al cierre de Agenda Base; PostgreSQL real operativo; 7/7 migraciones aplicadas; checkpoint E2E 1/1 aprobado.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agenda Base cerrada con 8/8 tareas Done, catálogo/disponibilidad operativos y checkpoint E2E real aprobado.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Mantener evidencia histórica del Sprint 4; Burndown reconstruido con evidencia Git/PR ya disponible.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">PostgreSQL activo; Prisma validado; fixtures E2E</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">R0.5</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sprint 5</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Citas y lista de espera</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Reserva, consulta y cancelación de citas; integración Web/API; lista de espera</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">HU-004/005/006 completadas; HU-007/008 backend implementadas; HU-021 Web de lista de espera/preferencias completada mediante PR #89. Validación: Web 56/56, development/seed 11/11 y Waitlist E2E 24/24.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Flujo núcleo de citas y lista de espera disponible y validado de punta a punta en Web + API + PostgreSQL.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Mantener evidencia histórica del Sprint 5 y continuar integración Web del motor de reasignación.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">HU-004/005/006; Auth; AgendaSlot; catálogos; PostgreSQL; apps/web; cliente HTTP centralizado; PR #43.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sprint 5 cerrado. HU-021 consolidó la experiencia Web de lista de espera y estabilizó el entorno local.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Criterios de interpretación del estado</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Entregable principal del Sprint disponible y verificable.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Avance alto</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Flujo de acceso y autorización base operativo y documentado</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Swagger/OpenAPI; rate limiting; controles de seguridad finales</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Config/env; PostgreSQL; roles/permisos</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">La seguridad base está implementada y ya es consumida por la aplicación web. Quedan documentación OpenAPI, controles finales de endurecimiento y pruebas específicas de seguridad/rendimiento.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R0.4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sprint 4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agenda base</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Instituciones, sedes, servicios, profesionales y disponibilidad read-only</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Catálogo institucional, servicios, profesionales y disponibilidad read-only; 69/69 pruebas unitarias al cierre de Agenda Base; PostgreSQL real operativo; 7/7 migraciones aplicadas; checkpoint E2E 1/1 aprobado.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agenda Base cerrada con 8/8 tareas Done, catálogo/disponibilidad operativos y checkpoint E2E real aprobado.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mantener evidencia histórica del Sprint 4; Burndown reconstruido con evidencia Git/PR ya disponible.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PostgreSQL activo; Prisma validado; fixtures E2E</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R0.5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sprint 5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Citas y lista de espera</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Reserva, consulta y cancelación de citas; integración Web/API; lista de espera</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">HU-004/005/006 completadas; HU-007/008 backend implementadas; HU-021 Web de lista de espera/preferencias completada mediante PR #89. Validación: Web 56/56, development/seed 11/11 y Waitlist E2E 24/24.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Flujo núcleo de citas y lista de espera disponible y validado de punta a punta en Web + API + PostgreSQL.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mantener evidencia histórica del Sprint 5 y continuar integración Web del motor de reasignación.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">HU-004/005/006; Auth; AgendaSlot; catálogos; PostgreSQL; apps/web; cliente HTTP centralizado; PR #43.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sprint 5 cerrado. HU-021 consolidó la experiencia Web de lista de espera y estabilizó el entorno local.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R0.6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sprint 6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Motor de reasignación y notificaciones internas</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Candidatos, ranking, ofertas, aceptación/rechazo, expiración automática, continuidad y centro de notificaciones</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">HU-009/010/011/016/018 backend; HU-022 Web ofertas; HU-023 expiración automática (PR #96, merge 109b1c9); HU-024 notificaciones internas (PR #99, merge b1bff30). Validación automática y manual PASS.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Motor de reasignación completo, expiración persistente, continuidad segura y notificaciones internas disponibles de punta a punta</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">MVP Web cerrado mediante HU-025/HU-026; mantener evidencia y preparar Sprint 7 / Desktop.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">HU-009/010/011/016/018; apps/web; runner de expiración; Notification; PostgreSQL</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sprint 6 cerrado. RF-029/RF-030/RF-034 quedan cubiertos. El backend continúa siendo fuente de verdad y las notificaciones externas permanecen fuera de alcance.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">R1.0</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sprint 8</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cierre MVP y preparación de defensa</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Web + escritorio + backend + BD + Docker + pruebas + documentación + presentación</x:t>
+    <x:t xml:space="preserve">Mayor parte del objetivo implementada; quedan cierres/evidencias.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Parcial</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Parte relevante implementada, pero faltan componentes obligatorios.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Pendiente</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">MVP end-to-end demostrable y entregables académicos completos</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cierre de Sprints anteriores</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Release académica final del proyecto.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Criterios de interpretación del estado</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Entregable principal del Sprint disponible y verificable.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Mayor parte del objetivo implementada; quedan cierres/evidencias.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Parcial</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Parte relevante implementada, pero faltan componentes obligatorios.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Trabajo aún no iniciado funcionalmente.</x:t>
   </x:si>
   <x:si>
@@ -261,42 +189,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Ruta de releases</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Análisis y arquitectura</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">→</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Base del proyecto</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Auth / RBAC operativos</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">8/8 tareas + E2E 1/1 + Burndown</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Citas y espera</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">HU-004–008 + HU-021 Web Done</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Reasignación + notificaciones</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">HU-022/023/024 Done · HU-025/026 cierre Web post-S6 Done</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cierre MVP</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cierre final y entregables restantes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Último avance incorporado</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -471,7 +363,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -537,6 +429,72 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -808,7 +766,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rda3fd3cfc2a74a05"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4e0928fefa1242e2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1058,7 +1016,7 @@
     </x:row>
     <x:row r="2" ht="39.75" customHeight="1">
       <x:c r="A2" s="15" t="str">
-        <x:v>Versión 1.8 · Fecha de corte: 23-09-2026 · Sprint 7 en progreso · HU-027 a HU-029 Done · Desktop/Tauri operativo con autenticación y gestión de sedes/servicios.</x:v>
+        <x:v>Versión 1.9 · Fecha de corte: 04-10-2026 · Sprint 7 cerrado · HU-001 a HU-038 Done · Sprint 8 planificado para integraciones externas · Sprint 9 reservado para cierre técnico y académico.</x:v>
       </x:c>
       <x:c r="B2" s="16"/>
       <x:c r="C2" s="16"/>
@@ -1134,97 +1092,97 @@
         <x:v>20</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="72" customHeight="1">
-      <x:c r="A6" s="1" t="str">
+    <x:row r="6" ht="70" customHeight="1">
+      <x:c r="A6" s="26" t="str">
         <x:v>R0.2</x:v>
       </x:c>
-      <x:c r="B6" s="1" t="str">
+      <x:c r="B6" s="26" t="str">
         <x:v>Sprint 2</x:v>
       </x:c>
-      <x:c r="C6" s="1" t="str">
+      <x:c r="C6" s="26" t="str">
         <x:v>Configuración técnica</x:v>
       </x:c>
-      <x:c r="D6" s="1" t="str">
+      <x:c r="D6" s="26" t="str">
         <x:v>Monorepo, backend base, PostgreSQL, Prisma, repositorio, Web y fundación Desktop</x:v>
       </x:c>
-      <x:c r="E6" s="1" t="str">
+      <x:c r="E6" s="26" t="str">
         <x:v>Avance alto</x:v>
       </x:c>
-      <x:c r="F6" s="1" t="str">
-        <x:v>Monorepo npm; NestJS; PostgreSQL; Prisma 7.10.0; migraciones; README; apps/web operativa; apps/desktop creada con Tauri 2 + React/Vite/TypeScript; @citajusta/client-core compartido; build y cargo check validados.</x:v>
-      </x:c>
-      <x:c r="G6" s="1" t="str">
-        <x:v>Entorno reproducible con clientes Web/Desktop base creados y conectables a la misma API</x:v>
-      </x:c>
-      <x:c r="H6" s="1" t="str">
-        <x:v>Completar Docker/Docker Compose y cierres técnicos restantes.</x:v>
-      </x:c>
-      <x:c r="I6" s="4" t="str">
+      <x:c r="F6" s="26" t="str">
+        <x:v>Monorepo npm; NestJS; PostgreSQL; Prisma 7.10.0; migraciones; README; apps/web operativa; apps/desktop Tauri 2 + React/Vite/TypeScript; @citajusta/client-core compartido; builds y cargo check validados.</x:v>
+      </x:c>
+      <x:c r="G6" s="26" t="str">
+        <x:v>Entorno reproducible con clientes Web/Desktop base creados y conectados a la misma API</x:v>
+      </x:c>
+      <x:c r="H6" s="26" t="str">
+        <x:v>Completar Docker/Docker Compose como parte del cierre técnico de Sprint 9.</x:v>
+      </x:c>
+      <x:c r="I6" s="29" t="str">
         <x:v>Node/npm; PostgreSQL; Rust/Cargo; MSVC Build Tools; WebView2</x:v>
       </x:c>
-      <x:c r="J6" s="4" t="str">
-        <x:v>La fundación Web y Desktop ya está disponible. La configuración técnica permanece en Avance alto porque contenedorización y cierres técnicos adicionales siguen pendientes.</x:v>
+      <x:c r="J6" s="29" t="str">
+        <x:v>La fundación Web y Desktop está disponible. La contenedorización se mantiene como cierre técnico planificado, no como requisito previo para las integraciones externas.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="72" customHeight="1">
-      <x:c r="A7" s="1" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B7" s="1" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C7" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="D7" s="1" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E7" s="1" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="F7" s="1" t="str">
-        <x:v>Registro/login/refresh/logout; Argon2id; sesiones; AccessTokenGuard; RBAC; contexto institucional; /users/me; Web protegida; Desktop autenticado con tokens sólo en memoria y cliente compartido. Regresión API al 23-09-2026: 394/394 PASS.</x:v>
-      </x:c>
-      <x:c r="G7" s="1" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="H7" s="1" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="I7" s="4" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="J7" s="4" t="s">
-        <x:v>29</x:v>
+      <x:c r="A7" s="26" t="str">
+        <x:v>R0.3</x:v>
+      </x:c>
+      <x:c r="B7" s="26" t="str">
+        <x:v>Sprint 3</x:v>
+      </x:c>
+      <x:c r="C7" s="26" t="str">
+        <x:v>Seguridad y usuarios</x:v>
+      </x:c>
+      <x:c r="D7" s="26" t="str">
+        <x:v>Auth, sesiones, JWT, RBAC, contexto institucional y validación</x:v>
+      </x:c>
+      <x:c r="E7" s="26" t="str">
+        <x:v>Avance alto</x:v>
+      </x:c>
+      <x:c r="F7" s="26" t="str">
+        <x:v>Registro/login/refresh/logout; Argon2id; sesiones; AccessTokenGuard; RBAC; AuthorizationContext; /users/me; Web protegida; Desktop autenticado y cliente compartido. Google OAuth/OIDC se planifica como método adicional en Sprint 8.</x:v>
+      </x:c>
+      <x:c r="G7" s="26" t="str">
+        <x:v>Flujo de acceso y autorización base operativo y documentado</x:v>
+      </x:c>
+      <x:c r="H7" s="26" t="str">
+        <x:v>Swagger/OpenAPI, rate limiting y hardening final quedan para Sprint 9; Google OAuth/OIDC se implementará en HU-040 sin reemplazar el login actual.</x:v>
+      </x:c>
+      <x:c r="I7" s="29" t="str">
+        <x:v>Config/env; PostgreSQL; roles/permisos; proveedores externos futuros</x:v>
+      </x:c>
+      <x:c r="J7" s="29" t="str">
+        <x:v>La seguridad base está implementada. Las integraciones externas deberán preservar RBAC, contexto institucional y manejo controlado de secretos.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="72" customHeight="1">
       <x:c r="A8" s="1" t="s">
-        <x:v>30</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="F8" s="1" t="s">
-        <x:v>34</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G8" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="H8" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="I8" s="4" t="s">
-        <x:v>37</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="J8" s="4" t="str">
         <x:v>Sprint 4 cerrado técnicamente con 8/8 tareas. Checkpoint E2E real 1/1 y Burndown histórico documentado. La regresión global API posterior alcanza 394/394 PASS.</x:v>
@@ -1232,135 +1190,167 @@
     </x:row>
     <x:row r="9" ht="72" customHeight="1">
       <x:c r="A9" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
-        <x:v>41</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="F9" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="G9" s="1" t="s">
-        <x:v>43</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="H9" s="1" t="s">
-        <x:v>44</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="I9" s="4" t="s">
-        <x:v>45</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="J9" s="4" t="s">
-        <x:v>46</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="72" customHeight="1">
-      <x:c r="A10" s="1" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B10" s="1" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C10" s="1" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="D10" s="1" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="E10" s="1" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F10" s="1" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="G10" s="1" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="H10" s="1" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="I10" s="4" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="J10" s="4" t="s">
-        <x:v>55</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="72" customHeight="1">
-      <x:c r="A11" s="1" t="str">
+        <x:v>37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="70" customHeight="1">
+      <x:c r="A10" s="26" t="str">
+        <x:v>R0.6</x:v>
+      </x:c>
+      <x:c r="B10" s="26" t="str">
+        <x:v>Sprint 6</x:v>
+      </x:c>
+      <x:c r="C10" s="26" t="str">
+        <x:v>Motor de reasignación y notificaciones internas</x:v>
+      </x:c>
+      <x:c r="D10" s="26" t="str">
+        <x:v>Candidatos, ranking, ofertas, aceptación/rechazo, expiración automática, continuidad y centro de notificaciones</x:v>
+      </x:c>
+      <x:c r="E10" s="26" t="str">
+        <x:v>Completo</x:v>
+      </x:c>
+      <x:c r="F10" s="26" t="str">
+        <x:v>HU-009/010/011/016/018 backend; HU-022 Web ofertas; HU-023 expiración automática (PR #96, merge 109b1c9); HU-024 notificaciones internas (PR #99, merge b1bff30). Validación automática y manual PASS.</x:v>
+      </x:c>
+      <x:c r="G10" s="26" t="str">
+        <x:v>Motor de reasignación completo, expiración persistente, continuidad segura y notificaciones internas disponibles de punta a punta</x:v>
+      </x:c>
+      <x:c r="H10" s="26" t="str">
+        <x:v>Mantener la evidencia histórica; los canales externos se formalizan como HU-039 Resend y HU-043 WhatsApp en Sprint 8.</x:v>
+      </x:c>
+      <x:c r="I10" s="29" t="str">
+        <x:v>HU-009/010/011/016/018; apps/web; runner de expiración; Notification; PostgreSQL</x:v>
+      </x:c>
+      <x:c r="J10" s="29" t="str">
+        <x:v>Sprint 6 cerrado. RF-029/RF-030/RF-034 quedan cubiertos. El backend sigue siendo fuente de verdad; los canales externos son adaptadores posteriores, no parte retroactiva del Sprint 6.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="78" customHeight="1">
+      <x:c r="A11" s="26" t="str">
         <x:v>R0.7</x:v>
       </x:c>
-      <x:c r="B11" s="1" t="str">
+      <x:c r="B11" s="26" t="str">
         <x:v>Sprint 7</x:v>
       </x:c>
-      <x:c r="C11" s="1" t="str">
-        <x:v>Aplicación institucional, operación y reportes</x:v>
-      </x:c>
-      <x:c r="D11" s="1" t="str">
-        <x:v>Desktop Tauri, autenticación institucional y módulos administrativos conectados a la API</x:v>
-      </x:c>
-      <x:c r="E11" s="1" t="str">
-        <x:v>En progreso</x:v>
-      </x:c>
-      <x:c r="F11" s="1" t="str">
-        <x:v>Backend HU-012/013/014/015/016/017/018/019/020 implementado. HU-027 fundó apps/desktop (PR #112, merge 6adab82); HU-028 agregó autenticación real + @citajusta/client-core (PR #113, merge ae151b3); HU-029 agregó gestión real de sedes/servicios (commit f58c742, merge e1cdb2e). Validación HU-029: API 394/394, E2E catálogo 15/15, Web 95/95, Desktop 16/16 y prueba manual Tauri/PostgreSQL PASS.</x:v>
-      </x:c>
-      <x:c r="G11" s="1" t="str">
-        <x:v>Aplicación de escritorio consume la API con autenticación/contexto real y permite avanzar progresivamente en la operación institucional principal</x:v>
-      </x:c>
-      <x:c r="H11" s="1" t="str">
-        <x:v>Refinar e implementar los siguientes módulos institucionales Desktop sin duplicar reglas del backend.</x:v>
-      </x:c>
-      <x:c r="I11" s="4" t="str">
+      <x:c r="C11" s="26" t="str">
+        <x:v>Aplicación institucional, operación, reportes y UX</x:v>
+      </x:c>
+      <x:c r="D11" s="26" t="str">
+        <x:v>Desktop Tauri operativo para catálogo, profesionales, agenda, disponibilidad, asistencia, reasignaciones, reportes y auditoría; mejora UX Web de ofertas</x:v>
+      </x:c>
+      <x:c r="E11" s="26" t="str">
+        <x:v>Completo</x:v>
+      </x:c>
+      <x:c r="F11" s="26" t="str">
+        <x:v>HU-027 fundación Desktop; HU-028 autenticación/client-core; HU-029 sedes/servicios; HU-030 profesionales; HU-031 agenda; HU-032 disponibilidad/bloqueos; HU-033 asistencia; HU-034 sistema visual; HU-035 UX ofertas Web; HU-036 supervisión de reasignaciones; HU-037 reportes; HU-038 auditoría. PR #135/#139/#141/#143/#147 y validaciones manuales/automáticas registradas.</x:v>
+      </x:c>
+      <x:c r="G11" s="26" t="str">
+        <x:v>Aplicación institucional consume la API con autenticación/contexto real y cubre los módulos Desktop previstos sin duplicar reglas del backend</x:v>
+      </x:c>
+      <x:c r="H11" s="26" t="str">
+        <x:v>Mantener evidencia Scrum y avanzar a Sprint 8 de integraciones externas.</x:v>
+      </x:c>
+      <x:c r="I11" s="29" t="str">
         <x:v>APIs institucionales; RBAC; AuthorizationContext; Tauri HTTP; @citajusta/client-core; PostgreSQL</x:v>
       </x:c>
-      <x:c r="J11" s="4" t="str">
-        <x:v>Sprint 7 activo. Desktop ya no es sólo una planificación: posee fundación nativa, autenticación real y primer módulo funcional. Profesionales, agenda, asistencia, reasignaciones, reportes y auditoría se conectarán progresivamente según historias refinadas.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="72" customHeight="1">
-      <x:c r="A12" s="1" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="B12" s="1" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="C12" s="1" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="D12" s="1" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="E12" s="1" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="F12" s="1" t="str">
-        <x:v>GitHub público; backend HU-001 a HU-020; HU-021 a HU-029 completadas; Web MVP cerrado; Desktop Tauri operativo con autenticación y gestión de sedes/servicios; PostgreSQL real; expiración automática, inicio automático de reasignación y notificaciones internas operativas.</x:v>
-      </x:c>
-      <x:c r="G12" s="1" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="H12" s="1" t="str">
-        <x:v>Completar módulos Desktop restantes; integraciones externas seleccionadas; Docker; OpenAPI; seguridad/rendimiento; documentación y defensa.</x:v>
-      </x:c>
-      <x:c r="I12" s="4" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="J12" s="4" t="s">
-        <x:v>63</x:v>
+      <x:c r="J11" s="29" t="str">
+        <x:v>Sprint 7 cerrado. HU-001 a HU-038 quedan Done; Desktop ya dispone de los módulos institucionales previstos y la Web recibió la modernización UX de ofertas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="82" customHeight="1">
+      <x:c r="A12" s="26" t="str">
+        <x:v>R0.8</x:v>
+      </x:c>
+      <x:c r="B12" s="26" t="str">
+        <x:v>Sprint 8</x:v>
+      </x:c>
+      <x:c r="C12" s="26" t="str">
+        <x:v>Integraciones externas</x:v>
+      </x:c>
+      <x:c r="D12" s="26" t="str">
+        <x:v>Resend, Google OAuth/OIDC, Google Calendar, Google Maps y WhatsApp condicionado</x:v>
+      </x:c>
+      <x:c r="E12" s="26" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="F12" s="26" t="str">
+        <x:v>HU-039 a HU-043 incorporadas al Product Backlog el 04-10-2026. Proveedores y orden de implementación definidos a nivel de planificación; sin afirmar integración funcional hasta su implementación y pruebas.</x:v>
+      </x:c>
+      <x:c r="G12" s="26" t="str">
+        <x:v>Integraciones seleccionadas operativas y seguras, preservando PostgreSQL/CitaJusta como fuente de verdad y sin ampliar permisos por identidad externa</x:v>
+      </x:c>
+      <x:c r="H12" s="26" t="str">
+        <x:v>Refinar e implementar HU-039–HU-043; configurar credenciales por entorno; validar consentimiento, privacidad, errores de proveedor y pruebas de integración.</x:v>
+      </x:c>
+      <x:c r="I12" s="29" t="str">
+        <x:v>Notificaciones internas; Auth/RBAC; citas; Branch; Google Cloud; Resend; decisión de proveedor WhatsApp</x:v>
+      </x:c>
+      <x:c r="J12" s="29" t="str">
+        <x:v>Orden previsto: Resend → Google OAuth/OIDC → Google Calendar → Google Maps → WhatsApp. WhatsApp permanece condicionado a proveedor, costos, consentimiento y plantillas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="82" customHeight="1">
+      <x:c r="A13" s="30" t="str">
+        <x:v>R1.0</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>Sprint 9</x:v>
+      </x:c>
+      <x:c r="C13" s="30" t="str">
+        <x:v>Cierre técnico y académico</x:v>
+      </x:c>
+      <x:c r="D13" s="30" t="str">
+        <x:v>Docker/Docker Compose, OpenAPI, hardening/rendimiento, documentación/evidencias y preparación de defensa</x:v>
+      </x:c>
+      <x:c r="E13" s="30" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="F13" s="30" t="str">
+        <x:v>Base funcional HU-001 a HU-038 Done; Sprint 8 de integraciones externas formalizado. Repositorio, PostgreSQL, Web y Desktop operativos como base del cierre.</x:v>
+      </x:c>
+      <x:c r="G13" s="30" t="str">
+        <x:v>Release académica end-to-end demostrable, reproducible y documentada con evidencias verificables</x:v>
+      </x:c>
+      <x:c r="H13" s="30" t="str">
+        <x:v>Completar Docker/Compose, Swagger/OpenAPI, controles finales de seguridad/rendimiento, documentación viva, matriz de evidencias, presentación y preparación de defensa.</x:v>
+      </x:c>
+      <x:c r="I13" s="30" t="str">
+        <x:v>Cierre de Sprint 8; infraestructura local; documentación Scrum/Capstone</x:v>
+      </x:c>
+      <x:c r="J13" s="30" t="str">
+        <x:v>Sprint 9 concentra cierres técnicos y académicos para evitar sobrecargar Sprint 8 con cinco integraciones externas más la entrega final.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="18" t="s">
-        <x:v>64</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B15" s="19"/>
       <x:c r="C15" s="19"/>
@@ -1377,39 +1367,39 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="10" t="s">
-        <x:v>65</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C16" s="10" t="s">
-        <x:v>25</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D16" s="10" t="s">
-        <x:v>66</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E16" s="1" t="s">
-        <x:v>67</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F16" s="10" t="s">
-        <x:v>68</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="G16" s="10" t="s">
-        <x:v>60</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="H16" s="10" t="s">
-        <x:v>69</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="I16" s="10" t="s">
-        <x:v>70</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="J16" s="10" t="s">
-        <x:v>71</x:v>
+        <x:v>47</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="142.5">
       <x:c r="A17" s="11" t="s">
-        <x:v>72</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B17" s="11" t="s">
-        <x:v>73</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C17" s="12"/>
       <x:c r="D17" s="12"/>
@@ -2447,7 +2437,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41fcfada8155466d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e6cd40518914592"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2466,7 +2456,7 @@
   <x:sheetData>
     <x:row r="1" ht="20.25">
       <x:c r="A1" s="21" t="str">
-        <x:v>CITAJUSTA — RESUMEN DEL RELEASE PLAN — ACTUALIZADO 23-09-2026</x:v>
+        <x:v>CITAJUSTA — RESUMEN DEL RELEASE PLAN — ACTUALIZADO 04-10-2026</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -2476,26 +2466,26 @@
     </x:row>
     <x:row r="3" ht="15">
       <x:c r="A3" s="2" t="s">
-        <x:v>74</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C3" s="5"/>
       <x:c r="D3" s="2" t="s">
-        <x:v>76</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E3" s="2" t="s">
-        <x:v>77</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="F3" s="5"/>
     </x:row>
     <x:row r="4" ht="28.5">
       <x:c r="A4" s="3" t="s">
-        <x:v>78</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B4" s="3" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C4" s="5"/>
       <x:c r="D4" s="3" t="s">
@@ -2503,20 +2493,20 @@
       </x:c>
       <x:c r="E4" s="3" t="n">
         <x:f t="shared" ref="E4:E8" si="0">B5</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F4" s="5"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="s">
-        <x:v>79</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B5" s="3" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C5" s="5"/>
       <x:c r="D5" s="3" t="s">
-        <x:v>25</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E5" s="3" t="n">
         <x:f t="shared" si="0"/>
@@ -2526,31 +2516,31 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="3" t="s">
-        <x:v>25</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B6" s="3" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C6" s="5"/>
       <x:c r="D6" s="3" t="s">
-        <x:v>72</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="E6" s="3" t="n">
         <x:f t="shared" si="0"/>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="5"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="3" t="s">
-        <x:v>72</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B7" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="5"/>
       <x:c r="D7" s="3" t="s">
-        <x:v>67</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E7" s="3" t="n">
         <x:f t="shared" si="0"/>
@@ -2560,27 +2550,27 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="3" t="s">
-        <x:v>80</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B8" s="3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="5"/>
       <x:c r="D8" s="4" t="s">
-        <x:v>60</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E8" s="4" t="n">
         <x:f t="shared" si="0"/>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F8" s="5"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="3" t="s">
-        <x:v>81</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B9" s="3" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C9" s="5"/>
       <x:c r="D9" s="5"/>
@@ -2589,10 +2579,10 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="5" t="s">
-        <x:v>82</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>23-09-2026</x:v>
+        <x:v>04-10-2026</x:v>
       </x:c>
       <x:c r="C10" s="5"/>
       <x:c r="D10" s="5"/>
@@ -2609,7 +2599,7 @@
     </x:row>
     <x:row r="12" ht="15">
       <x:c r="A12" s="22" t="s">
-        <x:v>83</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B12" s="16"/>
       <x:c r="C12" s="16"/>
@@ -2618,23 +2608,23 @@
       <x:c r="F12" s="17"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="4" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B13" s="4" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="C13" s="4" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D13" s="4" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E13" s="4" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="F13" s="4" t="s">
-        <x:v>86</x:v>
+      <x:c r="A13" s="4" t="str">
+        <x:v>R0.1</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>Análisis y arquitectura</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>Sprint 1</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>Completo</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>→</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>Base del proyecto</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2654,140 +2644,152 @@
         <x:v>→</x:v>
       </x:c>
       <x:c r="F14" s="4" t="str">
-        <x:v>Web + Desktop base operativos; Docker pendiente</x:v>
+        <x:v>Web + Desktop operativos; Docker en Sprint 9</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="4" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B15" s="4" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C15" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="D15" s="4" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E15" s="4" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="F15" s="4" t="s">
-        <x:v>87</x:v>
+      <x:c r="A15" s="4" t="str">
+        <x:v>R0.3</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="str">
+        <x:v>Seguridad y usuarios</x:v>
+      </x:c>
+      <x:c r="C15" s="4" t="str">
+        <x:v>Sprint 3</x:v>
+      </x:c>
+      <x:c r="D15" s="4" t="str">
+        <x:v>Avance alto</x:v>
+      </x:c>
+      <x:c r="E15" s="4" t="str">
+        <x:v>→</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>Auth / RBAC operativos; OIDC planificado Sprint 8</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="4" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="B16" s="4" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="C16" s="4" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="D16" s="4" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E16" s="4" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="F16" s="4" t="s">
-        <x:v>88</x:v>
+      <x:c r="A16" s="4" t="str">
+        <x:v>R0.4</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="str">
+        <x:v>Agenda base</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="str">
+        <x:v>Sprint 4</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="str">
+        <x:v>Completo</x:v>
+      </x:c>
+      <x:c r="E16" s="4" t="str">
+        <x:v>→</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>8/8 tareas + E2E 1/1 + Burndown</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="4" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B17" s="4" t="s">
-        <x:v>89</x:v>
-      </x:c>
-      <x:c r="C17" s="4" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D17" s="4" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E17" s="4" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="F17" s="4" t="s">
-        <x:v>90</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="28.5">
-      <x:c r="A18" s="4" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B18" s="4" t="s">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="C18" s="4" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="D18" s="4" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E18" s="4" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="F18" s="4" t="s">
-        <x:v>92</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="28.5">
-      <x:c r="A19" s="4" t="str">
+      <x:c r="A17" s="4" t="str">
+        <x:v>R0.5</x:v>
+      </x:c>
+      <x:c r="B17" s="4" t="str">
+        <x:v>Citas y espera</x:v>
+      </x:c>
+      <x:c r="C17" s="4" t="str">
+        <x:v>Sprint 5</x:v>
+      </x:c>
+      <x:c r="D17" s="4" t="str">
+        <x:v>Completo</x:v>
+      </x:c>
+      <x:c r="E17" s="4" t="str">
+        <x:v>→</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>HU-004–008 + HU-021 Web Done</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="38" customHeight="1">
+      <x:c r="A18" s="29" t="str">
+        <x:v>R0.6</x:v>
+      </x:c>
+      <x:c r="B18" s="29" t="str">
+        <x:v>Reasignación + notificaciones</x:v>
+      </x:c>
+      <x:c r="C18" s="29" t="str">
+        <x:v>Sprint 6</x:v>
+      </x:c>
+      <x:c r="D18" s="29" t="str">
+        <x:v>Completo</x:v>
+      </x:c>
+      <x:c r="E18" s="29" t="str">
+        <x:v>→</x:v>
+      </x:c>
+      <x:c r="F18" s="29" t="str">
+        <x:v>HU-022/023/024 Done · motor y notificaciones internas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="38" customHeight="1">
+      <x:c r="A19" s="29" t="str">
         <x:v>R0.7</x:v>
       </x:c>
-      <x:c r="B19" s="4" t="str">
-        <x:v>Aplicación institucional</x:v>
-      </x:c>
-      <x:c r="C19" s="4" t="str">
+      <x:c r="B19" s="29" t="str">
+        <x:v>Aplicación institucional + UX</x:v>
+      </x:c>
+      <x:c r="C19" s="29" t="str">
         <x:v>Sprint 7</x:v>
       </x:c>
-      <x:c r="D19" s="4" t="str">
-        <x:v>En progreso</x:v>
-      </x:c>
-      <x:c r="E19" s="4" t="str">
+      <x:c r="D19" s="29" t="str">
+        <x:v>Completo</x:v>
+      </x:c>
+      <x:c r="E19" s="29" t="str">
         <x:v>→</x:v>
       </x:c>
-      <x:c r="F19" s="4" t="str">
-        <x:v>Tauri + auth + Sedes/servicios Done; siguientes módulos por refinar</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="4" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="B20" s="4" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="C20" s="4" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="D20" s="4" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="E20" s="4" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="F20" s="4" t="s">
-        <x:v>94</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="15.75" customHeight="1">
-      <x:c r="A21" s="5"/>
-      <x:c r="B21" s="5"/>
-      <x:c r="C21" s="5"/>
-      <x:c r="D21" s="5"/>
-      <x:c r="E21" s="5"/>
-      <x:c r="F21" s="5"/>
+      <x:c r="F19" s="29" t="str">
+        <x:v>HU-027–038 Done; HU-035 UX Web incluida</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="38" customHeight="1">
+      <x:c r="A20" s="29" t="str">
+        <x:v>R0.8</x:v>
+      </x:c>
+      <x:c r="B20" s="29" t="str">
+        <x:v>Integraciones externas</x:v>
+      </x:c>
+      <x:c r="C20" s="29" t="str">
+        <x:v>Sprint 8</x:v>
+      </x:c>
+      <x:c r="D20" s="29" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="E20" s="29" t="str">
+        <x:v>→</x:v>
+      </x:c>
+      <x:c r="F20" s="29" t="str">
+        <x:v>HU-039–043: Resend, Google y WhatsApp condicionado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="38" customHeight="1">
+      <x:c r="A21" s="30" t="str">
+        <x:v>R1.0</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="str">
+        <x:v>Cierre técnico/académico</x:v>
+      </x:c>
+      <x:c r="C21" s="30" t="str">
+        <x:v>Sprint 9</x:v>
+      </x:c>
+      <x:c r="D21" s="30" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="E21" s="30" t="str">
+        <x:v>→</x:v>
+      </x:c>
+      <x:c r="F21" s="30" t="str">
+        <x:v>Docker + OpenAPI + hardening + docs + defensa</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
-      <x:c r="A22" s="23" t="s">
-        <x:v>95</x:v>
+      <x:c r="A22" s="23" t="str">
+        <x:v>Último avance: Sprint 7 cerrado; Sprint 8 integraciones externas; Sprint 9 cierre técnico/académico.</x:v>
       </x:c>
       <x:c r="B22" s="23"/>
       <x:c r="C22" s="23"/>
@@ -2796,9 +2798,7 @@
       <x:c r="F22" s="23"/>
     </x:row>
     <x:row r="23" ht="72" customHeight="1">
-      <x:c r="A23" s="24" t="str">
-        <x:v>Backend HU-001 a HU-020 completado. HU-021 a HU-026 cerraron el MVP Web. HU-027 creó la fundación Tauri (PR #112, 6adab82), HU-028 incorporó autenticación Desktop y @citajusta/client-core (PR #113, ae151b3), y HU-029 entregó gestión institucional de sedes/servicios (f58c742 → e1cdb2e). Sprint 7 continúa en progreso con el siguiente PBI Desktop pendiente de refinamiento.</x:v>
-      </x:c>
+      <x:c r="A23" s="24"/>
       <x:c r="B23" s="24"/>
       <x:c r="C23" s="24"/>
       <x:c r="D23" s="24"/>
@@ -3811,6 +3811,6 @@
     <x:mergeCell ref="A23:F26"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb0d77d524e740a6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R353f43a5cd9a4bd8"/>
 </x:worksheet>
 </file>
</xml_diff>